<commit_message>
chore(tool): Rebalancing_Tool_v4.0 Depotwert-Stand 18.08. (Owner-Pflege)
160 Zellen: Stichtag 15.06.->18.08., Depotwerte, abgeleitete Ist-Anteile
und Rebalancing-Hinweise (Gold 654->775 "Aufstocken", IWDA 3.943->7.459,
EIMI 1.350->3.604, EXUS 1.978->3.047 nach ING-Depotuebertrag).

Roster bleibt Juni-Stand: Adobe, Alphabet, Meta, Veeva und Costco fehlen,
die KYCCF-Zeile traegt provisorisch den VEEV-Wert (Owner-Workaround, um
das Tool nicht ohne Abstimmung umzubauen). Beides dokumentiert in
02_Analysen/2026-08-26_Depot-Reconciliation.md Abschnitt A.

§18.7 Smoke-Test PASS: 3 Sheets laden, 0 Error-Tokens, Formelzellen
340->340 (kein Verlust).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v4.0.xlsx
+++ b/03_Tools/Rebalancing_Tool_v4.0.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tobia\OneDrive\Desktop\Claude Stuff\03_Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46DB98B-56C7-4D88-ABB4-AF50664FF99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB611B10-B7F4-4AF1-A855-9326DF77AFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2082,7 +2082,7 @@
     <col min="10" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" customWidth="1"/>
     <col min="14" max="14" width="40.42578125" customWidth="1"/>
     <col min="15" max="15" width="116.42578125" customWidth="1"/>
     <col min="16" max="16" width="31.7109375" customWidth="1"/>
@@ -2113,7 +2113,7 @@
     <row r="2" spans="1:18" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="97">
         <f ca="1">TODAY()</f>
-        <v>46188</v>
+        <v>46252</v>
       </c>
       <c r="B2" s="96"/>
       <c r="C2" s="96"/>
@@ -2205,11 +2205,11 @@
         <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>654</v>
+        <v>775</v>
       </c>
       <c r="G5" s="6">
         <f t="shared" ref="G5:G24" si="0">IF(F$29=0,0,F5/F$29)</f>
-        <v>4.0149424616999663E-2</v>
+        <v>2.6054799125903513E-2</v>
       </c>
       <c r="H5" s="6">
         <f>VLOOKUP($B5,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2217,19 +2217,19 @@
       </c>
       <c r="I5" s="5">
         <f t="shared" ref="I5:I24" si="1">H5*F$29</f>
-        <v>805.76784675072747</v>
+        <v>1471.3821532492725</v>
       </c>
       <c r="J5" s="5">
         <f t="shared" ref="J5:J24" si="2">I5-F5</f>
-        <v>151.76784675072747</v>
+        <v>696.38215324927251</v>
       </c>
       <c r="K5" s="6">
         <f t="shared" ref="K5:K24" si="3">G5-H5</f>
-        <v>-9.3171127253863714E-3</v>
+        <v>-2.3411738216482521E-2</v>
       </c>
       <c r="L5" s="3" t="str">
         <f>IF(C5="Aktie",IF(K5&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K5&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K5&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
-        <v>⚖️ Halten</v>
+        <v>📈 Aufstocken</v>
       </c>
       <c r="M5" s="94" t="str">
         <f>IF(C5="Aktie",IF(G5&gt;'Parameter &amp; Regeln'!B$10,"🚨 ÜBER CAP","✅ OK"),"")</f>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="R5" s="89" t="str">
         <f>IF(AND(C5="Aktie",OR(LEFT(O5,1)="🔴",LEFT(N5,8)="DEFCON 1")),IF(J5&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J5&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J5&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🛒 Nachkaufen</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2267,11 +2267,11 @@
         <v>0.7</v>
       </c>
       <c r="F6" s="10">
-        <v>3943.46</v>
+        <v>7459</v>
       </c>
       <c r="G6" s="11">
         <f t="shared" si="0"/>
-        <v>0.24209120795130501</v>
+        <v>0.25076483442595393</v>
       </c>
       <c r="H6" s="6">
         <f>VLOOKUP($B6,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2279,15 +2279,15 @@
       </c>
       <c r="I6" s="10">
         <f t="shared" si="1"/>
-        <v>3254.6701260911736</v>
+        <v>5943.2298739088264</v>
       </c>
       <c r="J6" s="10">
         <f t="shared" si="2"/>
-        <v>-688.78987390882639</v>
+        <v>-1515.7701260911736</v>
       </c>
       <c r="K6" s="11">
         <f t="shared" si="3"/>
-        <v>4.228519437225553E-2</v>
+        <v>5.0958820846904451E-2</v>
       </c>
       <c r="L6" s="8" t="str">
         <f>IF(C6="Aktie",IF(K6&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K6&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K6&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2329,11 +2329,11 @@
         <v>0</v>
       </c>
       <c r="F7" s="10">
-        <v>1349.52</v>
+        <v>3604</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="0"/>
-        <v>8.2847785182161127E-2</v>
+        <v>0.12116322070936292</v>
       </c>
       <c r="H7" s="6">
         <f>VLOOKUP($B7,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2341,19 +2341,19 @@
       </c>
       <c r="I7" s="10">
         <f t="shared" si="1"/>
-        <v>1943.3224539282248</v>
+        <v>3548.6275460717748</v>
       </c>
       <c r="J7" s="10">
         <f t="shared" si="2"/>
-        <v>593.80245392822485</v>
+        <v>-55.372453928225241</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="3"/>
-        <v>-3.6453863702416947E-2</v>
+        <v>1.861571824784844E-3</v>
       </c>
       <c r="L7" s="8" t="str">
         <f>IF(C7="Aktie",IF(K7&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K7&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K7&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
-        <v>📈 Aufstocken</v>
+        <v>⚖️ Halten</v>
       </c>
       <c r="M7" s="12" t="str">
         <f>IF(C7="Aktie",IF(G7&gt;'Parameter &amp; Regeln'!B$10,"🚨 ÜBER CAP","✅ OK"),"")</f>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="R7" s="90" t="str">
         <f>IF(AND(C7="Aktie",OR(LEFT(O7,1)="🔴",LEFT(N7,8)="DEFCON 1")),IF(J7&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J7&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J7&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v>🛒 Nachkaufen</v>
+        <v/>
       </c>
     </row>
     <row r="8" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2391,11 +2391,11 @@
         <v>0</v>
       </c>
       <c r="F8" s="10">
-        <v>1978.17</v>
+        <v>3047</v>
       </c>
       <c r="G8" s="11">
         <f t="shared" si="0"/>
-        <v>0.12144095916607067</v>
+        <v>0.10243738443435872</v>
       </c>
       <c r="H8" s="6">
         <f>VLOOKUP($B8,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2403,15 +2403,15 @@
       </c>
       <c r="I8" s="10">
         <f t="shared" si="1"/>
-        <v>1295.5483026188167</v>
+        <v>2365.7516973811835</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" si="2"/>
-        <v>-682.62169738118337</v>
+        <v>-681.24830261881652</v>
       </c>
       <c r="K8" s="11">
         <f t="shared" si="3"/>
-        <v>4.1906526576351952E-2</v>
+        <v>2.2902951844640002E-2</v>
       </c>
       <c r="L8" s="8" t="str">
         <f>IF(C8="Aktie",IF(K8&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K8&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K8&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2453,11 +2453,11 @@
         <v>0.67</v>
       </c>
       <c r="F9" s="10">
-        <v>1366</v>
+        <v>2715</v>
       </c>
       <c r="G9" s="11">
         <f t="shared" si="0"/>
-        <v>8.3859501570063513E-2</v>
+        <v>9.1275844679778118E-2</v>
       </c>
       <c r="H9" s="6">
         <f>VLOOKUP($B9,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2465,15 +2465,15 @@
       </c>
       <c r="I9" s="10">
         <f t="shared" si="1"/>
-        <v>1295.5483026188167</v>
+        <v>2365.7516973811835</v>
       </c>
       <c r="J9" s="10">
         <f t="shared" si="2"/>
-        <v>-70.451697381183294</v>
+        <v>-349.24830261881652</v>
       </c>
       <c r="K9" s="11">
         <f t="shared" si="3"/>
-        <v>4.3250689803447928E-3</v>
+        <v>1.1741412090059397E-2</v>
       </c>
       <c r="L9" s="8" t="str">
         <f>IF(C9="Aktie",IF(K9&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K9&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K9&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K9&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="R9" s="90" t="str">
         <f>IF(AND(C9="Aktie",OR(LEFT(O9,1)="🔴",LEFT(N9,8)="DEFCON 1")),IF(J9&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J9&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J9&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>⏸️ Über Ziel</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2515,11 +2515,11 @@
         <v>0.62</v>
       </c>
       <c r="F10" s="10">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="G10" s="11">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5.8833417381072449E-3</v>
       </c>
       <c r="H10" s="6">
         <f>VLOOKUP($B10,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2527,15 +2527,15 @@
       </c>
       <c r="I10" s="10">
         <f t="shared" si="1"/>
-        <v>1137.5546071774975</v>
+        <v>2077.2453928225023</v>
       </c>
       <c r="J10" s="10">
         <f t="shared" si="2"/>
-        <v>1137.5546071774975</v>
+        <v>1902.2453928225023</v>
       </c>
       <c r="K10" s="11">
         <f t="shared" si="3"/>
-        <v>-6.9835111542192047E-2</v>
+        <v>-6.3951769804084804E-2</v>
       </c>
       <c r="L10" s="8" t="str">
         <f>IF(C10="Aktie",IF(K10&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K10&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K10&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2577,11 +2577,11 @@
         <v>0.68</v>
       </c>
       <c r="F11" s="10">
-        <v>193</v>
+        <v>362</v>
       </c>
       <c r="G11" s="11">
         <f t="shared" si="0"/>
-        <v>1.1848377601041184E-2</v>
+        <v>1.2170112623970416E-2</v>
       </c>
       <c r="H11" s="6">
         <f>VLOOKUP($B11,'Parameter &amp; Regeln'!$A$56:$B$62,2,FALSE)/'Parameter &amp; Regeln'!$B$4</f>
@@ -2589,15 +2589,15 @@
       </c>
       <c r="I11" s="10">
         <f t="shared" si="1"/>
-        <v>805.76784675072747</v>
+        <v>1471.3821532492725</v>
       </c>
       <c r="J11" s="10">
         <f t="shared" si="2"/>
-        <v>612.76784675072747</v>
+        <v>1109.3821532492725</v>
       </c>
       <c r="K11" s="11">
         <f t="shared" si="3"/>
-        <v>-3.7618159741344852E-2</v>
+        <v>-3.729642471841562E-2</v>
       </c>
       <c r="L11" s="13" t="str">
         <f>IF(C11="Aktie",IF(K11&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K11&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K11&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2639,11 +2639,11 @@
         <v>1</v>
       </c>
       <c r="F12" s="62">
-        <v>381</v>
+        <v>592</v>
       </c>
       <c r="G12" s="63">
         <f t="shared" si="0"/>
-        <v>2.3389802414490627E-2</v>
+        <v>1.990250462262565E-2</v>
       </c>
       <c r="H12" s="63">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -2651,15 +2651,15 @@
       </c>
       <c r="I12" s="62">
         <f t="shared" si="1"/>
-        <v>631.97478176527648</v>
+        <v>1154.0252182347238</v>
       </c>
       <c r="J12" s="62">
         <f t="shared" si="2"/>
-        <v>250.97478176527648</v>
+        <v>562.02521823472375</v>
       </c>
       <c r="K12" s="63">
         <f t="shared" si="3"/>
-        <v>-1.5407481775616069E-2</v>
+        <v>-1.8894779567481045E-2</v>
       </c>
       <c r="L12" s="60" t="str">
         <f>IF(C12="Aktie",IF(K12&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K12&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K12&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="R12" s="91" t="str">
         <f>IF(AND(C12="Aktie",OR(LEFT(O12,1)="🔴",LEFT(N12,8)="DEFCON 1")),IF(J12&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J12&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J12&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🚩 FLAG (gesperrt)</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2705,11 +2705,11 @@
         <v>1</v>
       </c>
       <c r="F13" s="64">
-        <v>378</v>
+        <v>398</v>
       </c>
       <c r="G13" s="78">
         <f t="shared" si="0"/>
-        <v>2.3205630741935584E-2</v>
+        <v>1.3380400067238191E-2</v>
       </c>
       <c r="H13" s="78">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2717,15 +2717,15 @@
       </c>
       <c r="I13" s="64">
         <f t="shared" si="1"/>
-        <v>284.38865179437437</v>
+        <v>519.31134820562556</v>
       </c>
       <c r="J13" s="64">
         <f t="shared" si="2"/>
-        <v>-93.611348205625632</v>
+        <v>121.31134820562556</v>
       </c>
       <c r="K13" s="78">
         <f t="shared" si="3"/>
-        <v>5.7468528563875722E-3</v>
+        <v>-4.0783778183098203E-3</v>
       </c>
       <c r="L13" s="76" t="str">
         <f>IF(C13="Aktie",IF(K13&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K13&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K13&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2771,11 +2771,11 @@
         <v>0</v>
       </c>
       <c r="F14" s="62">
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="G14" s="63">
         <f t="shared" si="0"/>
-        <v>3.4378712210274935E-2</v>
+        <v>1.9667170953101363E-2</v>
       </c>
       <c r="H14" s="63">
         <f>'Parameter &amp; Regeln'!$B$36/'Parameter &amp; Regeln'!$B$4</f>
@@ -2783,15 +2783,15 @@
       </c>
       <c r="I14" s="62">
         <f t="shared" si="1"/>
-        <v>505.57982541222111</v>
+        <v>923.22017458777884</v>
       </c>
       <c r="J14" s="62">
         <f t="shared" si="2"/>
-        <v>-54.420174587778888</v>
+        <v>338.22017458777884</v>
       </c>
       <c r="K14" s="63">
         <f t="shared" si="3"/>
-        <v>3.3408848581895807E-3</v>
+        <v>-1.1370656398983991E-2</v>
       </c>
       <c r="L14" s="60" t="str">
         <f>IF(C14="Aktie",IF(K14&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K14&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K14&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="R14" s="91" t="str">
         <f>IF(AND(C14="Aktie",OR(LEFT(O14,1)="🔴",LEFT(N14,8)="DEFCON 1")),IF(J14&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J14&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J14&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🛒 Nachkaufen</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2837,11 +2837,11 @@
         <v>1</v>
       </c>
       <c r="F15" s="64">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="G15" s="78">
         <f t="shared" si="0"/>
-        <v>2.7809922555811693E-2</v>
+        <v>1.5431164901664145E-2</v>
       </c>
       <c r="H15" s="78">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2849,15 +2849,15 @@
       </c>
       <c r="I15" s="64">
         <f t="shared" si="1"/>
-        <v>284.38865179437437</v>
+        <v>519.31134820562556</v>
       </c>
       <c r="J15" s="64">
         <f t="shared" si="2"/>
-        <v>-168.61134820562563</v>
+        <v>60.311348205625563</v>
       </c>
       <c r="K15" s="78">
         <f t="shared" si="3"/>
-        <v>1.0351144670263681E-2</v>
+        <v>-2.0276129838838666E-3</v>
       </c>
       <c r="L15" s="76" t="str">
         <f>IF(C15="Aktie",IF(K15&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K15&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K15&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2903,11 +2903,11 @@
         <v>1</v>
       </c>
       <c r="F16" s="62">
-        <v>481</v>
+        <v>470</v>
       </c>
       <c r="G16" s="63">
         <f t="shared" si="0"/>
-        <v>2.9528858166325438E-2</v>
+        <v>1.5800974953773743E-2</v>
       </c>
       <c r="H16" s="63">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -2915,15 +2915,15 @@
       </c>
       <c r="I16" s="62">
         <f t="shared" si="1"/>
-        <v>631.97478176527648</v>
+        <v>1154.0252182347238</v>
       </c>
       <c r="J16" s="62">
         <f t="shared" si="2"/>
-        <v>150.97478176527648</v>
+        <v>684.02521823472375</v>
       </c>
       <c r="K16" s="63">
         <f t="shared" si="3"/>
-        <v>-9.268426023781258E-3</v>
+        <v>-2.2996309236332953E-2</v>
       </c>
       <c r="L16" s="60" t="str">
         <f>IF(C16="Aktie",IF(K16&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K16&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K16&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="R16" s="91" t="str">
         <f>IF(AND(C16="Aktie",OR(LEFT(O16,1)="🔴",LEFT(N16,8)="DEFCON 1")),IF(J16&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J16&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J16&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🚩 FLAG (gesperrt)</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2969,11 +2969,11 @@
         <v>0</v>
       </c>
       <c r="F17" s="64">
-        <v>432</v>
+        <v>386</v>
       </c>
       <c r="G17" s="78">
         <f t="shared" si="0"/>
-        <v>2.652072084792638E-2</v>
+        <v>1.2976970919482265E-2</v>
       </c>
       <c r="H17" s="78">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -2981,15 +2981,15 @@
       </c>
       <c r="I17" s="64">
         <f t="shared" si="1"/>
-        <v>284.38865179437437</v>
+        <v>519.31134820562556</v>
       </c>
       <c r="J17" s="64">
         <f t="shared" si="2"/>
-        <v>-147.61134820562563</v>
+        <v>133.31134820562556</v>
       </c>
       <c r="K17" s="78">
         <f t="shared" si="3"/>
-        <v>9.0619429623783679E-3</v>
+        <v>-4.4818069660657461E-3</v>
       </c>
       <c r="L17" s="76" t="str">
         <f>IF(C17="Aktie",IF(K17&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K17&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K17&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K17&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3035,11 +3035,11 @@
         <v>0</v>
       </c>
       <c r="F18" s="62">
-        <v>0</v>
+        <v>561</v>
       </c>
       <c r="G18" s="63">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.8860312657589511E-2</v>
       </c>
       <c r="H18" s="63">
         <f>'Parameter &amp; Regeln'!$B$36/'Parameter &amp; Regeln'!$B$4</f>
@@ -3047,15 +3047,15 @@
       </c>
       <c r="I18" s="62">
         <f t="shared" si="1"/>
-        <v>505.57982541222111</v>
+        <v>923.22017458777884</v>
       </c>
       <c r="J18" s="62">
         <f t="shared" si="2"/>
-        <v>505.57982541222111</v>
+        <v>362.22017458777884</v>
       </c>
       <c r="K18" s="63">
         <f t="shared" si="3"/>
-        <v>-3.1037827352085354E-2</v>
+        <v>-1.2177514694495843E-2</v>
       </c>
       <c r="L18" s="60" t="str">
         <f>IF(C18="Aktie",IF(K18&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K18&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K18&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3101,11 +3101,11 @@
         <v>1</v>
       </c>
       <c r="F19" s="64">
-        <v>412</v>
+        <v>704</v>
       </c>
       <c r="G19" s="78">
         <f t="shared" si="0"/>
-        <v>2.5292909697559419E-2</v>
+        <v>2.3667843335014288E-2</v>
       </c>
       <c r="H19" s="78">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -3113,15 +3113,15 @@
       </c>
       <c r="I19" s="64">
         <f t="shared" si="1"/>
-        <v>631.97478176527648</v>
+        <v>1154.0252182347238</v>
       </c>
       <c r="J19" s="64">
         <f t="shared" si="2"/>
-        <v>219.97478176527648</v>
+        <v>450.02521823472375</v>
       </c>
       <c r="K19" s="78">
         <f t="shared" si="3"/>
-        <v>-1.3504374492547277E-2</v>
+        <v>-1.5129440855092408E-2</v>
       </c>
       <c r="L19" s="76" t="str">
         <f>IF(C19="Aktie",IF(K19&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K19&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K19&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="R19" s="92" t="str">
         <f>IF(AND(C19="Aktie",OR(LEFT(O19,1)="🔴",LEFT(N19,8)="DEFCON 1")),IF(J19&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J19&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J19&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🚩 FLAG (gesperrt)</v>
       </c>
     </row>
     <row r="20" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3167,11 +3167,11 @@
         <v>0</v>
       </c>
       <c r="F20" s="62">
-        <v>420</v>
+        <v>464</v>
       </c>
       <c r="G20" s="63">
         <f t="shared" si="0"/>
-        <v>2.5784034157706203E-2</v>
+        <v>1.559926037989578E-2</v>
       </c>
       <c r="H20" s="63">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -3179,15 +3179,15 @@
       </c>
       <c r="I20" s="62">
         <f t="shared" si="1"/>
-        <v>284.38865179437437</v>
+        <v>519.31134820562556</v>
       </c>
       <c r="J20" s="62">
         <f t="shared" si="2"/>
-        <v>-135.61134820562563</v>
+        <v>55.311348205625563</v>
       </c>
       <c r="K20" s="63">
         <f t="shared" si="3"/>
-        <v>8.3252562721581914E-3</v>
+        <v>-1.8595175056522317E-3</v>
       </c>
       <c r="L20" s="60" t="str">
         <f>IF(C20="Aktie",IF(K20&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K20&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K20&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3233,11 +3233,11 @@
         <v>1</v>
       </c>
       <c r="F21" s="64">
-        <v>954</v>
+        <v>4235</v>
       </c>
       <c r="G21" s="78">
         <f t="shared" si="0"/>
-        <v>5.8566591872504091E-2</v>
+        <v>0.14237687006219532</v>
       </c>
       <c r="H21" s="78">
         <f>'Parameter &amp; Regeln'!$B$35/'Parameter &amp; Regeln'!$B$4</f>
@@ -3245,23 +3245,23 @@
       </c>
       <c r="I21" s="64">
         <f t="shared" si="1"/>
-        <v>631.97478176527648</v>
+        <v>1154.0252182347238</v>
       </c>
       <c r="J21" s="64">
         <f t="shared" si="2"/>
-        <v>-322.02521823472352</v>
+        <v>-3080.974781765276</v>
       </c>
       <c r="K21" s="78">
         <f t="shared" si="3"/>
-        <v>1.9769307682397395E-2</v>
+        <v>0.10357958587208863</v>
       </c>
       <c r="L21" s="76" t="str">
         <f>IF(C21="Aktie",IF(K21&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K21&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K21&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K21&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
-        <v>⚖️ Halten</v>
+        <v>📉 Reduzieren</v>
       </c>
       <c r="M21" s="79" t="str">
         <f>IF(C21="Aktie",IF(G21&gt;'Parameter &amp; Regeln'!B$10,"🚨 ÜBER CAP","✅ OK"),"")</f>
-        <v>✅ OK</v>
+        <v>🚨 ÜBER CAP</v>
       </c>
       <c r="N21" s="82" t="s">
         <v>74</v>
@@ -3299,11 +3299,11 @@
         <v>1</v>
       </c>
       <c r="F22" s="62">
-        <v>396</v>
+        <v>490</v>
       </c>
       <c r="G22" s="63">
         <f t="shared" si="0"/>
-        <v>2.431066077726585E-2</v>
+        <v>1.6473356866700286E-2</v>
       </c>
       <c r="H22" s="63">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -3311,15 +3311,15 @@
       </c>
       <c r="I22" s="62">
         <f t="shared" si="1"/>
-        <v>284.38865179437437</v>
+        <v>519.31134820562556</v>
       </c>
       <c r="J22" s="62">
         <f t="shared" si="2"/>
-        <v>-111.61134820562563</v>
+        <v>29.311348205625563</v>
       </c>
       <c r="K22" s="63">
         <f t="shared" si="3"/>
-        <v>6.8518828917178386E-3</v>
+        <v>-9.8542101884772568E-4</v>
       </c>
       <c r="L22" s="60" t="str">
         <f>IF(C22="Aktie",IF(K22&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K22&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K22&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K22&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3365,11 +3365,11 @@
         <v>1</v>
       </c>
       <c r="F23" s="64">
-        <v>479</v>
+        <v>534</v>
       </c>
       <c r="G23" s="78">
         <f t="shared" si="0"/>
-        <v>2.9406077051288743E-2</v>
+        <v>1.7952597075138677E-2</v>
       </c>
       <c r="H23" s="78">
         <f>'Parameter &amp; Regeln'!$B$36/'Parameter &amp; Regeln'!$B$4</f>
@@ -3377,15 +3377,15 @@
       </c>
       <c r="I23" s="64">
         <f t="shared" si="1"/>
-        <v>505.57982541222111</v>
+        <v>923.22017458777884</v>
       </c>
       <c r="J23" s="64">
         <f t="shared" si="2"/>
-        <v>26.579825412221112</v>
+        <v>389.22017458777884</v>
       </c>
       <c r="K23" s="78">
         <f t="shared" si="3"/>
-        <v>-1.6317503007966111E-3</v>
+        <v>-1.3085230276946677E-2</v>
       </c>
       <c r="L23" s="76" t="str">
         <f>IF(C23="Aktie",IF(K23&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K23&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K23&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K23&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="R23" s="92" t="str">
         <f>IF(AND(C23="Aktie",OR(LEFT(O23,1)="🔴",LEFT(N23,8)="DEFCON 1")),IF(J23&gt;'Parameter &amp; Regeln'!$B$65,"🚩 FLAG (gesperrt)",""),IF(J23&gt;'Parameter &amp; Regeln'!$B$65,"🛒 Nachkaufen",IF(J23&lt;-'Parameter &amp; Regeln'!$B$65,"⏸️ Über Ziel","")))</f>
-        <v/>
+        <v>🛒 Nachkaufen</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3431,11 +3431,11 @@
         <v>1</v>
       </c>
       <c r="F24" s="62">
-        <v>428</v>
+        <v>699</v>
       </c>
       <c r="G24" s="63">
         <f t="shared" si="0"/>
-        <v>2.6275158617852987E-2</v>
+        <v>2.3499747856782653E-2</v>
       </c>
       <c r="H24" s="63">
         <f>'Parameter &amp; Regeln'!$B$37/'Parameter &amp; Regeln'!$B$4</f>
@@ -3443,15 +3443,15 @@
       </c>
       <c r="I24" s="62">
         <f t="shared" si="1"/>
-        <v>284.38865179437437</v>
+        <v>519.31134820562556</v>
       </c>
       <c r="J24" s="62">
         <f t="shared" si="2"/>
-        <v>-143.61134820562563</v>
+        <v>-179.68865179437444</v>
       </c>
       <c r="K24" s="63">
         <f t="shared" si="3"/>
-        <v>8.8163807323049757E-3</v>
+        <v>6.0409699712346415E-3</v>
       </c>
       <c r="L24" s="60" t="str">
         <f>IF(C24="Aktie",IF(K24&gt;'Parameter &amp; Regeln'!B$9,"📉 Reduzieren",IF(K24&lt;-'Parameter &amp; Regeln'!B$9,"📈 Aufstocken","⚖️ Halten")),IF(K24&gt;'Parameter &amp; Regeln'!B$8,"📉 Reduzieren",IF(K24&lt;-'Parameter &amp; Regeln'!B$8,"📈 Aufstocken","⚖️ Halten")))</f>
@@ -3490,11 +3490,11 @@
       <c r="E25" s="15"/>
       <c r="F25" s="16">
         <f>SUM(F5:F24)</f>
-        <v>15258.15</v>
+        <v>28714</v>
       </c>
       <c r="G25" s="17">
         <f>SUM(G5:G24)</f>
-        <v>0.93670633519858315</v>
+        <v>0.96533871238863656</v>
       </c>
       <c r="H25" s="17">
         <f>SUM(H5:H24)</f>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="I25" s="16">
         <f>SUM(I5:I24)</f>
-        <v>16289.15</v>
+        <v>29745.000000000004</v>
       </c>
       <c r="J25" s="16">
         <f>ROUND(SUM(J5:J24),2)</f>
@@ -3510,14 +3510,14 @@
       </c>
       <c r="K25" s="17">
         <f t="array" ref="K25">SUMPRODUCT((C5:C24="Aktie")*ABS(K5:K24))/COUNTIF(C5:C24,"Aktie")</f>
-        <v>1.1008731759278781E-2</v>
+        <v>1.666978639733966E-2</v>
       </c>
       <c r="L25" s="14" t="s">
         <v>86</v>
       </c>
       <c r="M25" s="18">
         <f>COUNTIF(M5:M24,"🚨 ÜBER CAP")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="19">
         <f>COUNTIF(N5:N24,"DEFCON 1*")+COUNTIF(N5:N24,"DEFCON 2*")+COUNTIF(N5:N24,"DEFCON 3*")</f>
@@ -3535,7 +3535,7 @@
     <row r="26" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K26" s="20">
         <f t="array" ref="K26">SUMPRODUCT((C5:C24&lt;&gt;"Aktie")*ABS(K5:K24))/COUNTIF(C5:C24,"&lt;&gt;Aktie")</f>
-        <v>3.4534433948613212E-2</v>
+        <v>3.0303527049338804E-2</v>
       </c>
       <c r="L26" s="21" t="s">
         <v>87</v>
@@ -3559,7 +3559,7 @@
         <v>91</v>
       </c>
       <c r="F27" s="26">
-        <v>74.3</v>
+        <v>143.22999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="F29" s="29">
         <f>F25 + F28</f>
-        <v>16289.15</v>
+        <v>29745</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="F31" s="67">
         <f>IF((F28-F30)&lt;=0,0,F27/(F28-F30))</f>
-        <v>0.11983870967741934</v>
+        <v>0.23101612903225804</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -3634,6 +3634,20 @@
   <conditionalFormatting sqref="H25">
     <cfRule type="expression" dxfId="17" priority="36">
       <formula>ABS($H$25-1)&gt;0.0001</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:K24">
+    <cfRule type="dataBar" priority="37">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BB3AE596-CA44-4F4A-94BC-647855B5C8CF}</x14:id>
+        </ext>
+      </extLst>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:L24">
@@ -3696,20 +3710,6 @@
       <formula>NOT(ISERROR(SEARCH("FLAG",R5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K24">
-    <cfRule type="dataBar" priority="37">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BB3AE596-CA44-4F4A-94BC-647855B5C8CF}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ungültiger Typ" error="Nur Gold, ETF oder Aktie erlaubt." sqref="C5:C24" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Gold,ETF,Aktie"</formula1>
@@ -3756,7 +3756,7 @@
   <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="C4" s="35">
         <f>'Portfolio &amp; Rebalancing'!F5</f>
-        <v>654</v>
+        <v>775</v>
       </c>
       <c r="D4" s="36">
         <f>'Portfolio &amp; Rebalancing'!E5</f>
@@ -3818,7 +3818,7 @@
       </c>
       <c r="C5" s="35">
         <f>'Portfolio &amp; Rebalancing'!F6</f>
-        <v>3943.46</v>
+        <v>7459</v>
       </c>
       <c r="D5" s="36">
         <f>'Portfolio &amp; Rebalancing'!E6</f>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="E5" s="35">
         <f t="shared" si="0"/>
-        <v>2760.422</v>
+        <v>5221.2999999999993</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="C6" s="35">
         <f>'Portfolio &amp; Rebalancing'!F7</f>
-        <v>1349.52</v>
+        <v>3604</v>
       </c>
       <c r="D6" s="36">
         <f>'Portfolio &amp; Rebalancing'!E7</f>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="C7" s="35">
         <f>'Portfolio &amp; Rebalancing'!F8</f>
-        <v>1978.17</v>
+        <v>3047</v>
       </c>
       <c r="D7" s="36">
         <f>'Portfolio &amp; Rebalancing'!E8</f>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="C8" s="35">
         <f>'Portfolio &amp; Rebalancing'!F9</f>
-        <v>1366</v>
+        <v>2715</v>
       </c>
       <c r="D8" s="36">
         <f>'Portfolio &amp; Rebalancing'!E9</f>
@@ -3892,7 +3892,7 @@
       </c>
       <c r="E8" s="35">
         <f t="shared" si="0"/>
-        <v>915.22</v>
+        <v>1819.0500000000002</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="C9" s="35">
         <f>'Portfolio &amp; Rebalancing'!F10</f>
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="D9" s="36">
         <f>'Portfolio &amp; Rebalancing'!E10</f>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="E9" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>108.5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="C10" s="35">
         <f>'Portfolio &amp; Rebalancing'!F11</f>
-        <v>193</v>
+        <v>362</v>
       </c>
       <c r="D10" s="36">
         <f>'Portfolio &amp; Rebalancing'!E11</f>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="E10" s="35">
         <f t="shared" si="0"/>
-        <v>131.24</v>
+        <v>246.16000000000003</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="C11" s="35">
         <f>'Portfolio &amp; Rebalancing'!F12</f>
-        <v>381</v>
+        <v>592</v>
       </c>
       <c r="D11" s="36">
         <f>'Portfolio &amp; Rebalancing'!E12</f>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="E11" s="35">
         <f t="shared" si="0"/>
-        <v>381</v>
+        <v>592</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="C12" s="35">
         <f>'Portfolio &amp; Rebalancing'!F13</f>
-        <v>378</v>
+        <v>398</v>
       </c>
       <c r="D12" s="36">
         <f>'Portfolio &amp; Rebalancing'!E13</f>
@@ -3980,7 +3980,7 @@
       </c>
       <c r="E12" s="35">
         <f t="shared" si="0"/>
-        <v>378</v>
+        <v>398</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="C13" s="35">
         <f>'Portfolio &amp; Rebalancing'!F14</f>
-        <v>560</v>
+        <v>585</v>
       </c>
       <c r="D13" s="36">
         <f>'Portfolio &amp; Rebalancing'!E14</f>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="C14" s="35">
         <f>'Portfolio &amp; Rebalancing'!F15</f>
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="D14" s="36">
         <f>'Portfolio &amp; Rebalancing'!E15</f>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="E14" s="35">
         <f t="shared" si="0"/>
-        <v>453</v>
+        <v>459</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="C15" s="35">
         <f>'Portfolio &amp; Rebalancing'!F16</f>
-        <v>481</v>
+        <v>470</v>
       </c>
       <c r="D15" s="36">
         <f>'Portfolio &amp; Rebalancing'!E16</f>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="E15" s="35">
         <f t="shared" si="0"/>
-        <v>481</v>
+        <v>470</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="C16" s="35">
         <f>'Portfolio &amp; Rebalancing'!F17</f>
-        <v>432</v>
+        <v>386</v>
       </c>
       <c r="D16" s="36">
         <f>'Portfolio &amp; Rebalancing'!E17</f>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="C17" s="35">
         <f>'Portfolio &amp; Rebalancing'!F18</f>
-        <v>0</v>
+        <v>561</v>
       </c>
       <c r="D17" s="36">
         <f>'Portfolio &amp; Rebalancing'!E18</f>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="C18" s="35">
         <f>'Portfolio &amp; Rebalancing'!F19</f>
-        <v>412</v>
+        <v>704</v>
       </c>
       <c r="D18" s="36">
         <f>'Portfolio &amp; Rebalancing'!E19</f>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="E18" s="35">
         <f t="shared" si="0"/>
-        <v>412</v>
+        <v>704</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="C19" s="35">
         <f>'Portfolio &amp; Rebalancing'!F20</f>
-        <v>420</v>
+        <v>464</v>
       </c>
       <c r="D19" s="36">
         <f>'Portfolio &amp; Rebalancing'!E20</f>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="C20" s="35">
         <f>'Portfolio &amp; Rebalancing'!F21</f>
-        <v>954</v>
+        <v>4235</v>
       </c>
       <c r="D20" s="36">
         <f>'Portfolio &amp; Rebalancing'!E21</f>
@@ -4156,7 +4156,7 @@
       </c>
       <c r="E20" s="35">
         <f t="shared" si="0"/>
-        <v>954</v>
+        <v>4235</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C21" s="35">
         <f>'Portfolio &amp; Rebalancing'!F22</f>
-        <v>396</v>
+        <v>490</v>
       </c>
       <c r="D21" s="36">
         <f>'Portfolio &amp; Rebalancing'!E22</f>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="E21" s="35">
         <f t="shared" si="0"/>
-        <v>396</v>
+        <v>490</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="C22" s="35">
         <f>'Portfolio &amp; Rebalancing'!F23</f>
-        <v>479</v>
+        <v>534</v>
       </c>
       <c r="D22" s="36">
         <f>'Portfolio &amp; Rebalancing'!E23</f>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="E22" s="35">
         <f t="shared" si="0"/>
-        <v>479</v>
+        <v>534</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C23" s="35">
         <f>'Portfolio &amp; Rebalancing'!F24</f>
-        <v>428</v>
+        <v>699</v>
       </c>
       <c r="D23" s="36">
         <f>'Portfolio &amp; Rebalancing'!E24</f>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="E23" s="35">
         <f t="shared" si="0"/>
-        <v>428</v>
+        <v>699</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -4232,11 +4232,11 @@
       </c>
       <c r="C24" s="38">
         <f>'Portfolio &amp; Rebalancing'!F25</f>
-        <v>15258.15</v>
+        <v>28714</v>
       </c>
       <c r="E24" s="38">
         <f>SUM(E4:E23)</f>
-        <v>8168.8819999999996</v>
+        <v>15976.009999999998</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B26" s="39">
         <f>IF('Portfolio &amp; Rebalancing'!F25=0,0,E24/'Portfolio &amp; Rebalancing'!F25)</f>
-        <v>0.53537827325068899</v>
+        <v>0.55638399387058568</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B27" s="39">
         <f>SUMPRODUCT('Portfolio &amp; Rebalancing'!$E$5:$E$24,'Portfolio &amp; Rebalancing'!$I$5:$I$24)/SUM('Portfolio &amp; Rebalancing'!$I$5:$I$24)</f>
-        <v>0.52614936954413194</v>
+        <v>0.52614936954413172</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="B14" s="45">
         <f>COUNTIFS('Portfolio &amp; Rebalancing'!A5:A24,"&lt;&gt;",'Portfolio &amp; Rebalancing'!F5:F24,"&gt;0")</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>